<commit_message>
Daily NSE scan: 2026-10-12
</commit_message>
<xml_diff>
--- a/output/2026-10-12/enriched_analysis.xlsx
+++ b/output/2026-10-12/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.266</v>
+        <v>2.253</v>
       </c>
       <c r="W2" t="n">
-        <v>2780</v>
+        <v>2796</v>
       </c>
       <c r="X2" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.885</v>
+        <v>0.878</v>
       </c>
       <c r="W3" t="n">
-        <v>915</v>
+        <v>922</v>
       </c>
       <c r="X3" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Y3" t="n">
         <v>47</v>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.046</v>
+        <v>0.044</v>
       </c>
       <c r="W4" t="n">
-        <v>2903</v>
+        <v>3016</v>
       </c>
       <c r="X4" t="n">
-        <v>9.98</v>
+        <v>10.4</v>
       </c>
       <c r="Y4" t="n">
         <v>36</v>
@@ -1625,10 +1625,10 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>1.867</v>
+        <v>1.93</v>
       </c>
       <c r="W5" t="n">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="n">
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>1.115</v>
+        <v>1.173</v>
       </c>
       <c r="W6" t="n">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="X6" t="n">
-        <v>7.64</v>
+        <v>7.24</v>
       </c>
       <c r="Y6" t="n">
         <v>17</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>1.188</v>
+        <v>1.199</v>
       </c>
       <c r="W7" t="n">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="X7" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="Y7" t="n">
         <v>22</v>
@@ -2322,10 +2322,10 @@
         <v>0.047</v>
       </c>
       <c r="W8" t="n">
-        <v>15198</v>
+        <v>15182</v>
       </c>
       <c r="X8" t="n">
-        <v>38.7</v>
+        <v>38.6</v>
       </c>
       <c r="Y8" t="n">
         <v>83</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.576</v>
+        <v>0.528</v>
       </c>
       <c r="W9" t="n">
-        <v>503</v>
+        <v>549</v>
       </c>
       <c r="X9" t="n">
-        <v>12.6</v>
+        <v>13.8</v>
       </c>
       <c r="Y9" t="n">
         <v>19</v>
@@ -2783,13 +2783,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>2.338</v>
+        <v>2.362</v>
       </c>
       <c r="W10" t="n">
-        <v>2511</v>
+        <v>2485</v>
       </c>
       <c r="X10" t="n">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="Y10" t="n">
         <v>6</v>
@@ -3021,7 +3021,7 @@
         <v>916</v>
       </c>
       <c r="X11" t="n">
-        <v>9.01</v>
+        <v>8.98</v>
       </c>
       <c r="Y11" t="n">
         <v>7</v>
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>0.052</v>
+        <v>0.05</v>
       </c>
       <c r="W12" t="n">
-        <v>1593</v>
+        <v>1654</v>
       </c>
       <c r="X12" t="n">
-        <v>21.4</v>
+        <v>22.3</v>
       </c>
       <c r="Y12" t="n">
         <v>55</v>
@@ -3482,10 +3482,10 @@
         <v>0.066</v>
       </c>
       <c r="W13" t="n">
-        <v>853</v>
+        <v>860</v>
       </c>
       <c r="X13" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="Y13" t="n">
         <v>19</v>
@@ -3709,10 +3709,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="W14" t="n">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="X14" t="n">
         <v>20.9</v>
@@ -3941,10 +3941,10 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>0.13</v>
+        <v>0.131</v>
       </c>
       <c r="W15" t="n">
-        <v>2412</v>
+        <v>2401</v>
       </c>
       <c r="X15" t="n">
         <v>21.1</v>
@@ -4176,10 +4176,10 @@
         <v>0.067</v>
       </c>
       <c r="W16" t="n">
-        <v>1663</v>
+        <v>1642</v>
       </c>
       <c r="X16" t="n">
-        <v>38.2</v>
+        <v>37.7</v>
       </c>
       <c r="Y16" t="n">
         <v>20</v>
@@ -4405,13 +4405,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.301</v>
+        <v>0.318</v>
       </c>
       <c r="W17" t="n">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="X17" t="n">
-        <v>25.5</v>
+        <v>24.1</v>
       </c>
       <c r="Y17" t="n">
         <v>12</v>
@@ -4637,13 +4637,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>3.014</v>
+        <v>3.051</v>
       </c>
       <c r="W18" t="n">
-        <v>653</v>
+        <v>645</v>
       </c>
       <c r="X18" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="Y18" t="n">
         <v>30</v>
@@ -4863,13 +4863,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.187</v>
+        <v>0.18</v>
       </c>
       <c r="W19" t="n">
-        <v>594</v>
+        <v>617</v>
       </c>
       <c r="X19" t="n">
-        <v>49.6</v>
+        <v>51.5</v>
       </c>
       <c r="Y19" t="n">
         <v>3</v>
@@ -5098,10 +5098,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W20" t="n">
-        <v>55024</v>
+        <v>54686</v>
       </c>
       <c r="X20" t="n">
-        <v>46.6</v>
+        <v>46.4</v>
       </c>
       <c r="Y20" t="n">
         <v>5</v>
@@ -5255,12 +5255,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hy-Tech Engineers Limited</t>
+          <t>Jayant Agro-Organics Limited</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -5272,101 +5272,107 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="G21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>212.86</v>
+      </c>
+      <c r="J21" t="n">
+        <v>232.74</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>67.13</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="N21" t="n">
+        <v>5704863</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>5704863</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S21" t="b">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
         <v>4</v>
       </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>90.37</v>
-      </c>
-      <c r="J21" t="n">
-        <v>68.68000000000001</v>
-      </c>
-      <c r="K21" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="L21" t="n">
-        <v>71.22</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="N21" t="n">
-        <v>8585000</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>8585000</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S21" t="b">
-        <v>0</v>
-      </c>
-      <c r="T21" t="n">
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="W21" t="n">
+        <v>633</v>
+      </c>
+      <c r="X21" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>-5</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>32</v>
+      </c>
+      <c r="AA21" t="n">
         <v>1</v>
       </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>29-09-2026</t>
-        </is>
-      </c>
-      <c r="V21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="W21" t="n">
-        <v>857</v>
-      </c>
-      <c r="X21" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>17</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>8.44</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>39</v>
-      </c>
       <c r="AB21" t="n">
-        <v>0.55</v>
+        <v>6.54</v>
       </c>
       <c r="AC21" t="n">
-        <v>23.9</v>
+        <v>14.8</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
       <c r="AE21" t="b">
         <v>1</v>
       </c>
       <c r="AF21" t="n">
-        <v>19.61</v>
-      </c>
-      <c r="AG21" t="inlineStr"/>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>226.38</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>205.68</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>10.8</v>
+      </c>
       <c r="AJ21" t="n">
-        <v>68.68000000000001</v>
+        <v>232.7375571148825</v>
       </c>
       <c r="AK21" t="n">
-        <v>31.6</v>
+        <v>-8.5</v>
       </c>
       <c r="AL21" t="inlineStr">
         <is>
@@ -5375,62 +5381,62 @@
       </c>
       <c r="AM21" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO21" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AQ21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR21" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AS21" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AW21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AX21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AY21" t="n">
         <v>0</v>
       </c>
       <c r="AZ21" t="n">
-        <v>8585000</v>
+        <v>0</v>
       </c>
       <c r="BA21" t="n">
-        <v>8585000</v>
+        <v>5704863</v>
       </c>
       <c r="BB21" t="n">
-        <v>8585000</v>
+        <v>5704863</v>
       </c>
       <c r="BC21" t="n">
-        <v>8585000</v>
+        <v>5704863</v>
       </c>
       <c r="BD21" t="n">
         <v>0</v>
@@ -5466,7 +5472,7 @@
         <v>0</v>
       </c>
       <c r="BO21" t="n">
-        <v>8585000</v>
+        <v>5704863</v>
       </c>
       <c r="BP21" t="n">
         <v>1</v>
@@ -5481,16 +5487,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jayant Agro-Organics Limited</t>
+          <t>Hy-Tech Engineers Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -5501,37 +5507,37 @@
         <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="G22" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>212.86</v>
+        <v>90.37</v>
       </c>
       <c r="J22" t="n">
-        <v>232.74</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>-8.5</v>
+        <v>31.6</v>
       </c>
       <c r="L22" t="n">
-        <v>67.13</v>
+        <v>71.22</v>
       </c>
       <c r="M22" t="n">
-        <v>0.57</v>
+        <v>0.86</v>
       </c>
       <c r="N22" t="n">
-        <v>5704863</v>
+        <v>8585000</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>5704863</v>
+        <v>8585000</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -5545,60 +5551,54 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.089</v>
+        <v>0.099</v>
       </c>
       <c r="W22" t="n">
-        <v>639</v>
+        <v>871</v>
       </c>
       <c r="X22" t="n">
-        <v>10.4</v>
+        <v>38</v>
       </c>
       <c r="Y22" t="n">
-        <v>-5</v>
+        <v>17</v>
       </c>
       <c r="Z22" t="n">
-        <v>32</v>
+        <v>8.44</v>
       </c>
       <c r="AA22" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="AB22" t="n">
-        <v>6.54</v>
+        <v>0.55</v>
       </c>
       <c r="AC22" t="n">
-        <v>14.8</v>
+        <v>23.9</v>
       </c>
       <c r="AD22" t="n">
-        <v>0.11</v>
+        <v>0.25</v>
       </c>
       <c r="AE22" t="b">
         <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>9</v>
-      </c>
-      <c r="AG22" t="n">
-        <v>226.38</v>
-      </c>
-      <c r="AH22" t="n">
-        <v>205.68</v>
-      </c>
-      <c r="AI22" t="n">
-        <v>10.8</v>
-      </c>
+        <v>19.61</v>
+      </c>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
       <c r="AJ22" t="n">
-        <v>232.7375571148825</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="AK22" t="n">
-        <v>-8.5</v>
+        <v>31.6</v>
       </c>
       <c r="AL22" t="inlineStr">
         <is>
@@ -5607,62 +5607,62 @@
       </c>
       <c r="AM22" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN22" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO22" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="AP22" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="AQ22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AR22" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="AS22" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="AT22" t="n">
         <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AW22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AX22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AY22" t="n">
         <v>0</v>
       </c>
       <c r="AZ22" t="n">
-        <v>0</v>
+        <v>8585000</v>
       </c>
       <c r="BA22" t="n">
-        <v>5704863</v>
+        <v>8585000</v>
       </c>
       <c r="BB22" t="n">
-        <v>5704863</v>
+        <v>8585000</v>
       </c>
       <c r="BC22" t="n">
-        <v>5704863</v>
+        <v>8585000</v>
       </c>
       <c r="BD22" t="n">
         <v>0</v>
@@ -5698,7 +5698,7 @@
         <v>0</v>
       </c>
       <c r="BO22" t="n">
-        <v>5704863</v>
+        <v>8585000</v>
       </c>
       <c r="BP22" t="n">
         <v>1</v>
@@ -5785,13 +5785,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>1.09</v>
+        <v>1.078</v>
       </c>
       <c r="W23" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="X23" t="n">
-        <v>5.32</v>
+        <v>5.38</v>
       </c>
       <c r="Y23" t="n">
         <v>31</v>
@@ -6013,13 +6013,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.391</v>
+        <v>0.403</v>
       </c>
       <c r="W24" t="n">
-        <v>1006</v>
+        <v>977</v>
       </c>
       <c r="X24" t="n">
-        <v>51.3</v>
+        <v>49.8</v>
       </c>
       <c r="Y24" t="n">
         <v>21</v>
@@ -6245,10 +6245,10 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.262</v>
+        <v>0.261</v>
       </c>
       <c r="W25" t="n">
-        <v>994</v>
+        <v>997</v>
       </c>
       <c r="X25" t="n">
         <v>27.1</v>
@@ -6477,13 +6477,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.13</v>
+        <v>0.127</v>
       </c>
       <c r="W26" t="n">
-        <v>615</v>
+        <v>632</v>
       </c>
       <c r="X26" t="n">
-        <v>13.5</v>
+        <v>13.9</v>
       </c>
       <c r="Y26" t="n">
         <v>-1</v>
@@ -6709,13 +6709,13 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.523</v>
+        <v>0.517</v>
       </c>
       <c r="W27" t="n">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="X27" t="n">
-        <v>35.4</v>
+        <v>35.8</v>
       </c>
       <c r="Y27" t="n">
         <v>21</v>
@@ -6941,10 +6941,10 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>1.893</v>
+        <v>1.876</v>
       </c>
       <c r="W28" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="n">
@@ -7171,13 +7171,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.042</v>
+        <v>0.041</v>
       </c>
       <c r="W29" t="n">
-        <v>1631</v>
+        <v>1672</v>
       </c>
       <c r="X29" t="n">
-        <v>21.3</v>
+        <v>21.9</v>
       </c>
       <c r="Y29" t="n">
         <v>10</v>
@@ -7403,13 +7403,13 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.532</v>
+        <v>0.504</v>
       </c>
       <c r="W30" t="n">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="X30" t="n">
-        <v>35.1</v>
+        <v>36.9</v>
       </c>
       <c r="Y30" t="n">
         <v>-44</v>
@@ -7635,13 +7635,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.26</v>
+        <v>0.255</v>
       </c>
       <c r="W31" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="X31" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="Y31" t="n">
         <v>16</v>
@@ -8093,13 +8093,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.232</v>
+        <v>0.236</v>
       </c>
       <c r="W33" t="n">
-        <v>1718</v>
+        <v>1690</v>
       </c>
       <c r="X33" t="n">
-        <v>18.2</v>
+        <v>17.9</v>
       </c>
       <c r="Y33" t="n">
         <v>-3</v>
@@ -8328,7 +8328,7 @@
         <v>0.043</v>
       </c>
       <c r="W34" t="n">
-        <v>3159</v>
+        <v>3149</v>
       </c>
       <c r="X34" t="n">
         <v>18.7</v>
@@ -8557,13 +8557,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.371</v>
+        <v>0.37</v>
       </c>
       <c r="W35" t="n">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="X35" t="n">
-        <v>93.2</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="Y35" t="n">
         <v>246</v>
@@ -8789,13 +8789,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.677</v>
+        <v>0.64</v>
       </c>
       <c r="W36" t="n">
-        <v>347</v>
+        <v>367</v>
       </c>
       <c r="X36" t="n">
-        <v>1120</v>
+        <v>1183</v>
       </c>
       <c r="Y36" t="n">
         <v>-61</v>
@@ -9017,13 +9017,13 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>0.863</v>
+        <v>0.835</v>
       </c>
       <c r="W37" t="n">
-        <v>3663</v>
+        <v>3786</v>
       </c>
       <c r="X37" t="n">
-        <v>25.6</v>
+        <v>26.5</v>
       </c>
       <c r="Y37" t="n">
         <v>2</v>
@@ -9252,10 +9252,10 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>5244</v>
+        <v>5337</v>
       </c>
       <c r="X38" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="Y38" t="n">
         <v>26</v>
@@ -9481,13 +9481,13 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0.105</v>
+        <v>0.101</v>
       </c>
       <c r="W39" t="n">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="X39" t="n">
-        <v>7.61</v>
+        <v>7.92</v>
       </c>
       <c r="Y39" t="n">
         <v>118</v>
@@ -9712,7 +9712,7 @@
         <v>0.011</v>
       </c>
       <c r="W40" t="n">
-        <v>4123</v>
+        <v>4134</v>
       </c>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="n">
@@ -9867,12 +9867,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>Hindcon Chemicals Limited</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -9884,40 +9884,40 @@
         </is>
       </c>
       <c r="E41" t="n">
+        <v>7</v>
+      </c>
+      <c r="F41" t="n">
         <v>4</v>
-      </c>
-      <c r="F41" t="n">
-        <v>8</v>
       </c>
       <c r="G41" t="n">
         <v>25</v>
       </c>
       <c r="H41" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>189.25</v>
+        <v>28.46</v>
       </c>
       <c r="J41" t="n">
-        <v>170.45</v>
+        <v>23.55</v>
       </c>
       <c r="K41" t="n">
-        <v>11</v>
+        <v>20.8</v>
       </c>
       <c r="L41" t="n">
-        <v>67.54000000000001</v>
+        <v>68.34</v>
       </c>
       <c r="M41" t="n">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="N41" t="n">
-        <v>2560187</v>
+        <v>2018403</v>
       </c>
       <c r="O41" t="n">
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>2560187</v>
+        <v>2018403</v>
       </c>
       <c r="Q41" t="n">
         <v>0</v>
@@ -9931,94 +9931,94 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="V41" t="n">
-        <v>0.1</v>
+        <v>0.146</v>
       </c>
       <c r="W41" t="n">
-        <v>255</v>
+        <v>138</v>
       </c>
       <c r="X41" t="n">
-        <v>27.2</v>
+        <v>32</v>
       </c>
       <c r="Y41" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="Z41" t="n">
-        <v>1.87</v>
+        <v>3.17</v>
       </c>
       <c r="AA41" t="n">
-        <v>-31</v>
+        <v>7</v>
       </c>
       <c r="AB41" t="n">
-        <v>3.36</v>
+        <v>0.49</v>
       </c>
       <c r="AC41" t="n">
-        <v>4.96</v>
+        <v>8.76</v>
       </c>
       <c r="AD41" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AE41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF41" t="n">
-        <v>2.97</v>
+        <v>14.87</v>
       </c>
       <c r="AG41" t="n">
-        <v>182.38</v>
+        <v>24.83</v>
       </c>
       <c r="AH41" t="n">
-        <v>164.81</v>
+        <v>22.86</v>
       </c>
       <c r="AI41" t="n">
-        <v>31.2</v>
+        <v>22.8</v>
       </c>
       <c r="AJ41" t="n">
-        <v>170.4518641810919</v>
+        <v>23.5472893358377</v>
       </c>
       <c r="AK41" t="n">
-        <v>11</v>
+        <v>20.9</v>
       </c>
       <c r="AL41" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN41" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO41" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="AP41" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="AQ41" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="AR41" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="AS41" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="AT41" t="n">
         <v>0</v>
@@ -10027,13 +10027,13 @@
         <v>0</v>
       </c>
       <c r="AV41" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AW41" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="AX41" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="AY41" t="n">
         <v>0</v>
@@ -10042,13 +10042,13 @@
         <v>0</v>
       </c>
       <c r="BA41" t="n">
-        <v>0</v>
+        <v>1308280</v>
       </c>
       <c r="BB41" t="n">
-        <v>2560187</v>
+        <v>2018403</v>
       </c>
       <c r="BC41" t="n">
-        <v>2560187</v>
+        <v>2018403</v>
       </c>
       <c r="BD41" t="n">
         <v>0</v>
@@ -10084,10 +10084,10 @@
         <v>0</v>
       </c>
       <c r="BO41" t="n">
-        <v>0</v>
+        <v>1308280</v>
       </c>
       <c r="BP41" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="BQ41" t="n">
         <v>0</v>
@@ -10099,16 +10099,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Hindcon Chemicals Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -10116,40 +10116,40 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G42" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>28.46</v>
+        <v>365.05</v>
       </c>
       <c r="J42" t="n">
-        <v>23.55</v>
+        <v>338.1</v>
       </c>
       <c r="K42" t="n">
-        <v>20.8</v>
+        <v>8</v>
       </c>
       <c r="L42" t="n">
-        <v>68.34</v>
+        <v>66.73</v>
       </c>
       <c r="M42" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="N42" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="O42" t="n">
         <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
@@ -10163,69 +10163,69 @@
         <v>0</v>
       </c>
       <c r="T42" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.138</v>
+        <v>0.076</v>
       </c>
       <c r="W42" t="n">
-        <v>146</v>
+        <v>444</v>
       </c>
       <c r="X42" t="n">
-        <v>33.6</v>
+        <v>13.1</v>
       </c>
       <c r="Y42" t="n">
-        <v>19</v>
+        <v>-8</v>
       </c>
       <c r="Z42" t="n">
-        <v>3.17</v>
+        <v>24</v>
       </c>
       <c r="AA42" t="n">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="AB42" t="n">
-        <v>0.49</v>
+        <v>14.36</v>
       </c>
       <c r="AC42" t="n">
-        <v>8.76</v>
+        <v>9.94</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="AE42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF42" t="n">
-        <v>14.87</v>
+        <v>18</v>
       </c>
       <c r="AG42" t="n">
-        <v>24.83</v>
+        <v>370.99</v>
       </c>
       <c r="AH42" t="n">
-        <v>22.86</v>
+        <v>275.33</v>
       </c>
       <c r="AI42" t="n">
-        <v>22.8</v>
+        <v>60.2</v>
       </c>
       <c r="AJ42" t="n">
-        <v>23.5472893358377</v>
+        <v>338.1</v>
       </c>
       <c r="AK42" t="n">
-        <v>20.9</v>
+        <v>8</v>
       </c>
       <c r="AL42" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="AM42" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Stale Accumulation</t>
         </is>
       </c>
       <c r="AN42" t="inlineStr">
@@ -10235,22 +10235,22 @@
       </c>
       <c r="AO42" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AP42" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AQ42" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="AR42" t="n">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="AS42" t="n">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="AT42" t="n">
         <v>0</v>
@@ -10259,13 +10259,13 @@
         <v>0</v>
       </c>
       <c r="AV42" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AW42" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="AX42" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AY42" t="n">
         <v>0</v>
@@ -10274,13 +10274,13 @@
         <v>0</v>
       </c>
       <c r="BA42" t="n">
-        <v>1308280</v>
+        <v>0</v>
       </c>
       <c r="BB42" t="n">
-        <v>2018403</v>
+        <v>0</v>
       </c>
       <c r="BC42" t="n">
-        <v>2018403</v>
+        <v>3381000</v>
       </c>
       <c r="BD42" t="n">
         <v>0</v>
@@ -10316,10 +10316,10 @@
         <v>0</v>
       </c>
       <c r="BO42" t="n">
-        <v>1308280</v>
+        <v>0</v>
       </c>
       <c r="BP42" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="BQ42" t="n">
         <v>0</v>
@@ -10331,57 +10331,57 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
+        <v>24</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>8</v>
+      </c>
+      <c r="G43" t="n">
         <v>25</v>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" t="n">
-        <v>15</v>
-      </c>
-      <c r="G43" t="n">
-        <v>17</v>
-      </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I43" t="n">
-        <v>365.05</v>
+        <v>189.25</v>
       </c>
       <c r="J43" t="n">
-        <v>338.1</v>
+        <v>170.45</v>
       </c>
       <c r="K43" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L43" t="n">
-        <v>66.73</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M43" t="n">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="N43" t="n">
-        <v>3381000</v>
+        <v>2560187</v>
       </c>
       <c r="O43" t="n">
         <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>3381000</v>
+        <v>2560187</v>
       </c>
       <c r="Q43" t="n">
         <v>0</v>
@@ -10395,94 +10395,94 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.079</v>
+        <v>0.097</v>
       </c>
       <c r="W43" t="n">
-        <v>430</v>
+        <v>265</v>
       </c>
       <c r="X43" t="n">
-        <v>12.7</v>
+        <v>28.4</v>
       </c>
       <c r="Y43" t="n">
-        <v>-8</v>
+        <v>24</v>
       </c>
       <c r="Z43" t="n">
-        <v>24</v>
+        <v>1.87</v>
       </c>
       <c r="AA43" t="n">
-        <v>33</v>
+        <v>-31</v>
       </c>
       <c r="AB43" t="n">
-        <v>14.36</v>
+        <v>3.36</v>
       </c>
       <c r="AC43" t="n">
-        <v>9.94</v>
+        <v>4.96</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="AE43" t="b">
         <v>1</v>
       </c>
       <c r="AF43" t="n">
-        <v>18</v>
+        <v>2.97</v>
       </c>
       <c r="AG43" t="n">
-        <v>370.99</v>
+        <v>182.38</v>
       </c>
       <c r="AH43" t="n">
-        <v>275.33</v>
+        <v>164.81</v>
       </c>
       <c r="AI43" t="n">
-        <v>60.2</v>
+        <v>31.2</v>
       </c>
       <c r="AJ43" t="n">
-        <v>338.1</v>
+        <v>170.4518641810919</v>
       </c>
       <c r="AK43" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="AL43" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM43" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN43" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AQ43" t="n">
         <v>0</v>
       </c>
       <c r="AR43" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="AS43" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="AT43" t="n">
         <v>0</v>
@@ -10494,10 +10494,10 @@
         <v>0</v>
       </c>
       <c r="AW43" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AX43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY43" t="n">
         <v>0</v>
@@ -10509,10 +10509,10 @@
         <v>0</v>
       </c>
       <c r="BB43" t="n">
-        <v>0</v>
+        <v>2560187</v>
       </c>
       <c r="BC43" t="n">
-        <v>3381000</v>
+        <v>2560187</v>
       </c>
       <c r="BD43" t="n">
         <v>0</v>
@@ -10551,7 +10551,7 @@
         <v>0</v>
       </c>
       <c r="BP43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BQ43" t="n">
         <v>0</v>
@@ -10635,10 +10635,10 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.051</v>
+        <v>0.052</v>
       </c>
       <c r="W44" t="n">
-        <v>958</v>
+        <v>945</v>
       </c>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="n">
@@ -10868,10 +10868,10 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>3656</v>
+        <v>3740</v>
       </c>
       <c r="X45" t="n">
-        <v>82.3</v>
+        <v>84.2</v>
       </c>
       <c r="Y45" t="n">
         <v>42</v>
@@ -11100,7 +11100,7 @@
         <v>0.006</v>
       </c>
       <c r="W46" t="n">
-        <v>4839</v>
+        <v>4860</v>
       </c>
       <c r="X46" t="n">
         <v>12.5</v>
@@ -11328,10 +11328,10 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>103712</v>
+        <v>102815</v>
       </c>
       <c r="X47" t="n">
-        <v>29.9</v>
+        <v>29.6</v>
       </c>
       <c r="Y47" t="n">
         <v>18</v>
@@ -11557,13 +11557,13 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.234</v>
+        <v>0.236</v>
       </c>
       <c r="W48" t="n">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="X48" t="n">
-        <v>22.8</v>
+        <v>22.6</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>
@@ -12454,70 +12454,70 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hy-Tech Engineers Limited</t>
+          <t>Jayant Agro-Organics Limited</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>90.37</v>
+        <v>212.86</v>
       </c>
       <c r="D21" t="n">
-        <v>68.68000000000001</v>
+        <v>232.74</v>
       </c>
       <c r="E21" t="n">
-        <v>31.6</v>
+        <v>-8.5</v>
       </c>
       <c r="F21" t="n">
-        <v>71.22</v>
+        <v>67.13</v>
       </c>
       <c r="G21" t="n">
-        <v>0.86</v>
+        <v>0.57</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jayant Agro-Organics Limited</t>
+          <t>Hy-Tech Engineers Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>212.86</v>
+        <v>90.37</v>
       </c>
       <c r="D22" t="n">
-        <v>232.74</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>-8.5</v>
+        <v>31.6</v>
       </c>
       <c r="F22" t="n">
-        <v>67.13</v>
+        <v>71.22</v>
       </c>
       <c r="G22" t="n">
-        <v>0.57</v>
+        <v>0.86</v>
       </c>
       <c r="H22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
     </row>
@@ -13154,105 +13154,105 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>Hindcon Chemicals Limited</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>189.25</v>
+        <v>28.46</v>
       </c>
       <c r="D41" t="n">
-        <v>170.45</v>
+        <v>23.55</v>
       </c>
       <c r="E41" t="n">
-        <v>11</v>
+        <v>20.8</v>
       </c>
       <c r="F41" t="n">
-        <v>67.54000000000001</v>
+        <v>68.34</v>
       </c>
       <c r="G41" t="n">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Hindcon Chemicals Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>28.46</v>
+        <v>365.05</v>
       </c>
       <c r="D42" t="n">
-        <v>23.55</v>
+        <v>338.1</v>
       </c>
       <c r="E42" t="n">
-        <v>20.8</v>
+        <v>8</v>
       </c>
       <c r="F42" t="n">
-        <v>68.34</v>
+        <v>66.73</v>
       </c>
       <c r="G42" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="H42" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>365.05</v>
+        <v>189.25</v>
       </c>
       <c r="D43" t="n">
-        <v>338.1</v>
+        <v>170.45</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F43" t="n">
-        <v>66.73</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G43" t="n">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>